<commit_message>
📊 محتوى @ahmed_alshuhail — 2026-06-07
</commit_message>
<xml_diff>
--- a/content/ahmed_alshuhail/2026-06-07/ahmed_alshuhail_2026-06-07.xlsx
+++ b/content/ahmed_alshuhail/2026-06-07/ahmed_alshuhail_2026-06-07.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="74">
   <si>
     <t>م</t>
   </si>
@@ -47,6 +47,351 @@
     <t>ملاحظات</t>
   </si>
   <si>
+    <t>٧‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t>نصائح استثمارية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍الأراضي الزراعية حول حمى المدينة
+▪️الأراضي الزراعية تتفاعل سعرياً بشكل إيجابي لو صدر تحويلها سكنياً، وتتفاعل أكثر وأكثر لو صدر ما يقرر بقاءها زراعياً، بل قد ترتفع لمستويات تاريخية لو قُرر ذلك على مدد معينة وبتنظيم معين في التطوير الريفي
+▪️عدد الأراضي الزراعية في مدينة الرياض على أساس 20,000م² لكل قطعة أرض لا يصل إلى 65,000 أرض في أفضل سيناريو على محيط 10 كيلو من أطراف المدينة من كل اتجاه، وهذا السيناريو الأفضل على الورق، ويستحيل حدوثه، لذا التقديرات أقل من ذلك بكثير، وأقل القليل في الشمال الغربي وعلى حمى وادي صفار وما حوله وما فوقه وما تحته
+▪️لا نرى توسعاً في الاستثمار الزراعي والريفي الفاخر لغرض إعادة البيع بسبب عدم وجود البيئة التشريعية المتكاملة والناضجة، والتي تحتاج تكاتف العديد من الوزارات والهيئات
+▪️أطلع على نموذج توسكانا بإيطاليا، ونموذج بروفانس بفرنسا، ونموذج ساتوياما باليابان، وأنا لا أتفق ولا أختلف مع هذه النماذج بقدر أهمية بناء بيئة استثمارية وتعزيز للهوية الحضرية تعكس تطور المدينة وتخلق نطاقاً واسعاً من الرغبات والاهتمامات
+▪️أشير إلى أن ضريبة الأراضي الزراعية مطبقة في العديد من دول العالم، ولكن غالباً ما ترتبط بأهداف تنموية مقابل دعم يحقق نتائج مؤكدة في الإنتاج
+▪️أختم بأن المؤشرات تقول أنه بحلول عام 2050م سيكون في الرياض 3.5 مليون متقاعد و 120,000 مليونير كسيناريو متوسط وهذا يجب أن يستعوب بشكل عميق ويحلل بشكل أعمق
+هذا والله أعلم، والله من وراء القصد</t>
+  </si>
+  <si>
+    <t>الأراضي الزراعية المحيطة بالمدن الكبرى كالرياض تمثل فرصة استثمارية مركّبة تستوجب فهماً عميقاً قبل الدخول فيها؛ فهي ترتفع قيمتها سواء أُعيد تصنيفها سكنياً أو بقيت زراعية ضمن منظومة تطوير ريفي منظّم، وهذا يعكس ندرة حقيقية في المعروض إذ لا يتجاوز عدد القطع الزراعية المحيطة بأطراف الرياض في أفضل التقديرات 65,000 قطعة. والمشكلة الجوهرية اليوم أن البيئة التشريعية لم تنضج بعد لاستيعاب الاستثمار الزراعي والريفي الفاخر، وهو ما يتطلب تنسيقاً حقيقياً بين الجهات الحكومية. والأهم أن المستثمر الواعي عليه أن يضع في حسبانه أن الرياض مقبلة بحلول 2050م على بيئة ديموغرافية واقتصادية استثنائية، مما يعني أن الأراضي ذات الطابع الريفي الفاخر ستكون من أكثر الأصول العقارية جاذبية لشريحة المتقاعدين وأصحاب الثروات المتنامية، وهذا يستوجب من المطورين والمستثمرين التفكير الاستراتيجي المبكر قبل أن تُحسم المعادلة التشريعية والتنموية.</t>
+  </si>
+  <si>
+    <t>لم ينشر</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t xml:space="preserve">📍ـ X خدم 18 سنة قي الشركة Y
+1️⃣ راتبه عند الاستقالة 25,000﷼
+2️⃣ حقوقه 387,500﷼
+3️⃣ يستحق تقاعد مبكر بعد 10 سنوات
+4️⃣ يرغب بالاشتراك الاختياري
+5️⃣ الشريحة رقم 34 الأقرب لراتبه
+6️⃣ مقدار الشريحة 26,200﷼
+7️⃣ ليس لديه رغبة بزيادة سنوية 
+8️⃣ سيدفع إجمالي 565,920﷼
+9️⃣ دفعات على 120 شهر (10 سنوات)
+🔟 شهرياً 4,716﷼ = 18% من 6️⃣☝️
+📍السؤال:
+▪️أين يستثمر 387,500﷼ (حقوقه)
+▪️لسداد الاشتراك = 565,920﷼
+▪️يحتاج آمن 100% :
+1️⃣ استثمار بمتوسط 8.4% سنوياً مركباً
+2️⃣ ليتمكن من سحب 4,716﷼ شهرياً</t>
+  </si>
+  <si>
+    <t>موظف أمضى 18 عاماً في خدمة شركته وقرر الاستقالة براتب 25,000 ريال، فاستحق مكافأة نهاية خدمة بلغت 387,500 ريال. الآن أمامه خيار الاشتراك الاختياري في التأمينات الاجتماعية لضمان تقاعد مبكر بعد 10 سنوات، وذلك بدفع 4,716 ريالاً شهرياً لمدة 120 شهراً، أي ما مجموعه 565,920 ريالاً. السؤال الجوهري: كيف يُشغّل مكافأته البالغة 387,500 ريال لتغطية هذا الالتزام كاملاً؟ الجواب في الاستثمار العقاري، إذ يُعدّ من أكثر القنوات أماناً وعائداً في المملكة، فالعقار المدروس يحقق عوائد إيجارية تتراوح بين 7% و10% سنوياً بشكل مركب، ما يُمكّنه من سحب دفعته الشهرية دون المساس برأس المال، بل وتنميته على المدى البعيد. الاستثمار العقاري ليس ترفاً، بل هو الخيار الأذكى لمن يسعى لتحويل حقوقه المالية إلى دخل ثابت ومستدام.</t>
+  </si>
+  <si>
+    <t>توعية عقارية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ماشاء تبارك الله 
+الحمدالله على كثير فضله</t>
+  </si>
+  <si>
+    <t>نعمة التملك العقاري من أعظم النعم التي يمن بها الله على عباده، فامتلاك المسكن الملائم يمنح الفرد الاستقرار النفسي والأسري الذي لا يعادله شيء. واليوم مع تطور منظومة الإسكان في المملكة وتوسع خيارات التمويل العقاري الميسر، باتت فرصة التملك أكثر قرباً من أي وقت مضى، فاغتنم الفرصة ولا تُؤخر قرارك.</t>
+  </si>
+  <si>
+    <t>٦‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍فرصة للاستثمار مع @Sukuk_SA
+▪️مساهمة راز الماسية العقاري
+▪️تطرح غدا 7 يونيو الساعة 1مساءً
+،،،
+1️⃣ المطور مساهم بـ 16%
+2️⃣ عائد الاستثمار المتوقع 38.09% 
+3️⃣ خلال مدة متوقعة 24 شهرًا ☝️
+4️⃣ المطور متخصص في مدينة جدة
+5️⃣ الطور باع أكثر من 1,000 وحدة
+6️⃣ العقار في حي مميز وموقع أميز:
+▪️حي السلامة
+▪️ تقاطع طريق المدينة مع طريق حراء
+7️⃣ نقطة رقم 1️⃣ يدفعها المطور أولاً
+،،،
+* ساهم لتنويع مصادر الاستثمار 👍
+* لتحميل التطبيق: 
+https://t.co/t6G1Xo39tL</t>
+  </si>
+  <si>
+    <t>من أبرز معايير تقييم فرص الاستثمار العقاري: نسبة مساهمة المطور في المشروع، إذ تعكس ثقته الفعلية بجدوى العائد. مساهمة راز الماسية العقاري المطروحة عبر منصة صكوك تجمع عدة مؤشرات إيجابية؛ مطور متخصص في السوق الجداوي بسجل تجاوز ألف وحدة مباعة، وموقع في حي السلامة عند تقاطع طريق المدينة مع طريق حراء وهو من المواقع ذات الطلب المرتفع. العائد المتوقع 38% خلال 24 شهراً، مع التزام المطور بسداد حصته أولاً مما يُعزز الثقة في الجدية. تنويع مصادر الدخل عبر الاستثمار العقاري المدروس ركيزة مالية يوصي بها المختصون، وتقييم أي فرصة يبدأ بفهم هيكلها المالي وخلفية المطور قبل اتخاذ القرار.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍م. عبدالله الحماد:
+▪️"المضاربات صارت من الماضي"
+▪️التصريح قبل 6 أشهر
+،،،
+📍🔻 المضاربات 73% في حي الخير
+▪️المصدر: @paseetah
+،،،
+📍مقارنة ¼ من 25 مع ¼ من 26:
+1️⃣ ¼ 2025: 1070 صفقة مكررة
+2️⃣ ¼ 2026: 294 صفقة مكررة
+▪️انخفاض الصفقات المكررة 73%
+3️⃣ ¼ 2025: متوسط م² 2300﷼
+4️⃣ ¼ 2026: متوسط م² 1360﷼
+▪️انخفاض المتوسط المتر² 59%</t>
+  </si>
+  <si>
+    <t>من أبرز المؤشرات التي ينبغي للمستثمر العقاري متابعتها: نسبة الصفقات المكررة في أي حي، إذ تعكس مستوى المضاربة وتقلبات السوق. بيانات حي الخير تكشف انخفاضاً حاداً في الصفقات المكررة بلغ 73% بين الربع الأول من 2025 والربع الأول من 2026، وتراجعاً في متوسط سعر المتر المربع من 2300 ريال إلى 1360 ريال، أي بانخفاض يقارب 59%. هذا النوع من البيانات يؤكد أن السوق في مراحل تصحيح حقيقية، وأن قراءة المؤشرات الكمية قبل اتخاذ أي قرار شراء أو بيع ليست ترفاً بل ضرورة. المستثمر الواعي لا يبني قراره على التصريحات، بل على الأرقام.</t>
+  </si>
+  <si>
+    <t>٤‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍مرفق مواقع المواقف المرصفة
+▪️عددها حدود 2700 موقف
+،،،
+1️⃣ الذكاء الاصطناعي عبر البث المباشر قادر على قياس الأشغال و وقت الذروة ومتوسط مدة التوقف
+2️⃣ مدينة الرياض قادرة على ضخ 1.5 مليون موقف على الشوارع التجارية لكن فعلياً لا يمكن إدارة وتشغيل أكثر من 200 ألف موقف وفق محاكاة عالية المدخلات مع الذكاء الاصطتاعي 
+3️⃣ يقول الذكاء الاصطناعي أن @Riyadh_Parking قد تربح قرابة 1 مليار إذا أدارت 100 ألف موقف بكفاءة و صلاحيات أوسع ويمكن تحقيق ذلك بحلول 2031م</t>
+  </si>
+  <si>
+    <t>تُعدّ إدارة مواقف السيارات من أكثر القطاعات العقارية المدرّة للدخل إذا أُحسن توظيف التقنية في تشغيلها. تشير التحليلات المدعومة بالذكاء الاصطناعي إلى أن مدينة الرياض تمتلك طاقة استيعابية تتجاوز مليونًا ونصف موقف على شوارعها التجارية، غير أن الطاقة الفعلية القابلة للإدارة الكفؤة لا تتعدى مئتي ألف موقف. والأهم من ذلك أن إدارة مئة ألف موقف فقط بمنظومة ذكية متكاملة قد تُدرّ عائدًا يقترب من مليار ريال، وهو ما يكشف حجم الفرص الاستثمارية المهدرة في البنية التحتية العقارية للمدن. إن استثمار المواقف لم يعد خدمةً مساندة، بل بات أصلًا عقاريًا حقيقيًا يستحق الدراسة والتخطيط الاستراتيجي.</t>
+  </si>
+  <si>
+    <t>٣‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍في أزمة كورونا أخذت توصية من أخي ثامر، أدام الله ظله، وهي:
+▪️يجب أن تعرف بشكل مفصل كيف نمت المدن المليونية، وكيف تطورت بنيتها التحتية، وكيف أن اقتصاد الفرد يخلق الفرص العقارية، وأن اقتصاد الدولة يخلق الاستدامة العمرانية في تلك المدن التي حققت نموًا في التوسع سكانيا وجغرافيا، وعليه فإن ذلك وقود التأمل والاستقراء والتنبؤ والاستشراف الجيد لمستقبل المدينة</t>
+  </si>
+  <si>
+    <t>من أعمق الدروس في الاستثمار العقاري أن تفهم كيف تنمو المدن الكبرى، وكيف تتشكّل بنيتها التحتية عبر الزمن، فاقتصاد الفرد هو من يصنع الفرص العقارية اليومية، بينما اقتصاد الدولة هو الضامن للاستدامة العمرانية على المدى البعيد. المستثمر الناجح لا يشتري عقاراً، بل يشتري مستقبل مدينة، وذلك لا يتحقق إلا بدراسة معمّقة لأنماط التوسع السكاني والجغرافي، واستقراء المؤشرات التي تحكم حركة المدن قبل أن تتحرك الأسعار.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍تذبذب وارتباك في الأسعار
+تحليل أبو سعد وليس تحليلي 🙏
+▪️التسعير مرتبك، وأشار إلى أن الفارق بين حي القيروان وحي المهدية أقل من 2000 ﷼ للمتر² كمتوسط، وهذا مؤشر لاقتناص الفرص ومؤشر للتخارج في الوقت نفسه ، وأنه في أواخر 2017م حصل مثل ذلك الأمر لمن تخارج من حي عرقة واشترى في حي الملقا، مع تحفظه أن يحدث نفس السيناريو في النمو نظراً للإرادة السياسية لتحقيق التوازن الذي لا مفر منه
+▪️حي السليمانية أصبح أغلى من حي العارض، والمروج أغلى من حي الغدير لأي أرض تكون الأطوال فيها مناسبة للتطوير لعدة وحدات مشتركة، كما أن حي العقيق أصبح مربحاً أكثر للمطورين وأكثر أماناً من حي النرجس
+▪️ختم كلامه لي بأمر صادم للغاية، فيقول: كلما أتخارج أكون أكثر حياداً وتصوراً في رؤية توجه العقار، ولم تسعفني خبرتي الطويلة في الاكتناز لفهم توجه العقار بدقه وإنما أنا في ركب النمو الاقتصادي الذي انتفعت منه ولم ينتفع مني، حيث أن أعظم الإمبراطوريات العقارية التي عمرها أقل من ربع قرن هي نتيجة تدوير الأموال وبناء هندسة تمويلية مع البنوك والصناديق، وللأسف الاكتناز يؤلمني من الداخل، حيث إنني أتألم عندما أجلس مع عقاريين مطورين لديهم 100 موظف، فضلاً عن 1000 موظف، وأنا لدي وكيل واحد بلا راتب، ومنفعته في مناصفة السعي مع الوسطاء، (شكرته على صراحته)
+،،،
+أبو سعد رجل يحبنا ونحبه ونصاحبه لكسب الدنيا وكسب الآخرة، حيث أني أجاهده على فضل الوقف وأٌشربه في عقله كما تشرب الإسفنجة من الماء، وهذه غايتي وأمنيتي ورجائي ومنتهى أملي، والله من وراء القصد</t>
+  </si>
+  <si>
+    <t>من أبرز ما يُلفت الانتباه في سوق الرياض اليوم أن الفوارق السعرية بين الأحياء باتت تتقارب بشكل لافت؛ إذ يكاد الفارق بين بعض الأحياء الراقية والأحياء المجاورة لها لا يتجاوز ألفي ريال للمتر المربع، وهو ما يُمثّل في آنٍ واحد فرصة للدخول وإشارة للخروج، تماماً كما حدث في 2017 حين تقاربت أسعار أحياء متعددة ثم تباينت مساراتها لاحقاً. والمتأمل في السوق اليوم يجد أن معادلة التقييم تغيّرت؛ فثمة أحياء تجاوزت في أسعارها أحياءً كانت تُعدّ الأعلى تاريخياً. والدرس العقاري الأعمق هنا أن تدوير رأس المال وبناء هندسة تمويلية محكمة أثبتا قدرةً على بناء الثروة أسرع من الاكتناز، غير أن المستثمر الواعي يُوازن بين العائد المادي وأثره الاجتماعي، ولعل توجيه جزء من هذه الثروة نحو الوقف العقاري خيرٌ يدوم ويتجاوز حدود الأرباح.</t>
+  </si>
+  <si>
+    <t>٢‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t>أشكركم وجزاكم الله عنا خير الجزاء</t>
+  </si>
+  <si>
+    <t>نتوجه بخالص الشكر والتقدير لكل من وثق بنا وأسهم في نشر الوعي العقاري، فالمجتمع المثقف عقارياً هو الأساس لاتخاذ قرارات سليمة تحمي حقوق الجميع وتُعزز الاستقرار في السوق. ونؤكد أن رسالتنا مستمرة في تقديم المعلومة الصحيحة والمحتوى الموثوق الذي يُمكّن كل فرد من التعامل مع العقار بوعي ودراية.</t>
+  </si>
+  <si>
+    <t>▪️صاحبي الي يحدثني عن نيته عنده فوق نصف مليون متابع ودائما موفق وأظن أن ذلك من حسن نيته والله أعلم https://t.co/cESBicAtPJ</t>
+  </si>
+  <si>
+    <t>من أهم العوامل التي تصنع النجاح في مجال العقارات هي النية الصادقة والشفافية التامة مع العملاء، فالمتخصص الناجح لا يبني سمعته على الإعلانات والمظاهر، بل على ثقة من تعامل معه وصدق توصياته. العقار استثمار طويل الأمد، والمستشار الأمين الذي يضع مصلحة العميل فوق عمولته هو من يستحق الثقة ويدوم نجاحه.</t>
+  </si>
+  <si>
+    <t>تمويل عقاري</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍العقد التمويلي = ورقة مالية
+▪️مرفق طريقة مبسطة للتوضيح والتقريب لكيفية تداول عقود التمويل العقاري المرهونة كورقة مالية، وهو تصور لغير الماليين والتطبيق الفعلي مختلف وفق سياسات وتفاصيل موسعة
+1️⃣ 1,000 عقد تمويلي عقاري
+2️⃣ كل عقد بـ مليون﷼
+3️⃣ فائدة كل تمويل 700 ألف﷼
+4️⃣ مدة التمويل 20 سنة لكل عقد
+5️⃣ العقود تمت 12 سنة دون تعثر
+6️⃣ عند 12 سنة استرد أصل التمويل
+7️⃣ قيمة كل عقار اليوم 1.5 مليون﷼
+▪️وفق المعطيات ☝️:
+1️⃣ كل عقد متبقي عليه 700 ألف﷼
+2️⃣ أي: كل العقود 700 مليون﷼
+3️⃣ قيمة كل عقار 1.5 مليون﷼
+4️⃣ أي: قيمة كل العقارات بـ 1.5 مليار﷼
+5️⃣ اشتر 1,000 عقد تمويلي 
+6️⃣ بقيمة 500 مليون﷼ نقداً
+7️⃣ سوف تستردها 700 مليون﷼
+8️⃣ ستردها الاسترداد 8 سنوات
+9️⃣ الفائدة 40% (5% سنوي كمتوسط)
+🔟 الضمان 1.5 مليار مقابل 500 مليون</t>
+  </si>
+  <si>
+    <t>هل تعلم أن عقود التمويل العقاري يمكن أن تُتداول كورقة مالية؟ تخيّل مجموعة من ألف عقد تمويلي، كل عقد بمليون ريال ومدته عشرون عاماً، وقد اكتمل منها اثنا عشر عاماً دون أي تعثر. في هذه الحالة، يبقى على كل عقد نحو سبعمائة ألف ريال، أي ما مجموعه سبعمائة مليون ريال، فيما ارتفعت قيمة العقارات الضامنة لتبلغ مليار وخمسمائة مليون ريال. هنا يكمن جوهر الفرصة: شراء هذه العقود بخمسمائة مليون ريال نقداً يعني استرداد سبعمائة مليون خلال ثماني سنوات بعائد يبلغ أربعين بالمئة، مع ضمان عقاري يفوق قيمة الاستثمار بثلاثة أضعاف. هذا النموذج يوضح كيف تتحول الأصول العقارية إلى أدوات مالية قابلة للتداول، وهو ما يُعرف بالتوريق العقاري الذي يُسهم في تعميق السوق المالي وتوفير السيولة اللازمة لتمويل مزيد من المشاريع السكنية.</t>
+  </si>
+  <si>
+    <t>١‏/٦‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍التمويل العقاري (2026م)
+▪️ما يعلن من @SAMA_GOV من أرقام يُصاغ خبره وفق رغبة وتوجه الكاتب، سواء في صحيفة أو "تغريدة" وحتى تستوعب الأرقام، سوف أخرج عن المألوف من المقارنة الشهرية أو الربعية أو المماثلة التي تحكمها العادة الإحصائية، فضلا عن الظروف الزمانية والسوقية
+▪️عند مقارنة أول 4 أشهر للأعوام 2024م و2025م و2026م لتمويل العقارات للأفراد:
+1️⃣ 2024م = 22.87 مليار﷼
+2️⃣ 2025م = 28.39 مليار﷼
+3️⃣ 2026م = 16.33 مليار﷼
+ـ أي أن:
+▪️التمويل العقاري السكني للأفراد خلال أول 4 أشهر من 2026م كان أقل بـ34% مقارنة بالفترة نفسها من 2025م
+▪️السوق فقد نحو 11.77 مليار﷼ من التمويلات الجديدة مقارنة بأول 4 أشهر من 2025م، وهو تراجع يوضح لك الركود
+📍توضيح إضافي:
+▪️ارتفاع متوسط الفائدة من 3.5% في أول 4 أشهر من 2025م إلى 4% في أول 4 أشهر من 2026م لا يخفض القدرة الشرائية بنسبة 0.5% فقط، بل "قد" يخفض قيمة العقار التي يستطيع الفرد شراءها بنحو 4% إلى 6% تقريباً، بحسب مدة التمويل والراتب والقسط الشهري، لذا فإن أثر ذلك على الطلب العقاري يكون أكبر من الزيادة الظاهرة في نسبة الفائدة
+▪️أوصي شركات التطوير العقاري باستيعاب ذلك جيداً، والاستمرار في مرونة التسعير ومواكبة المرحلة
+،،،
+والله يعلم ونحن لا نعلم 
+والله من وراء القصد</t>
+  </si>
+  <si>
+    <t>بيانات البنك المركزي تكشف تراجعاً لافتاً في التمويل العقاري للأفراد خلال أول أربعة أشهر من 2026م، إذ بلغ نحو 16.33 مليار ريال مقارنةً بـ28.39 مليار في الفترة ذاتها من 2025م، أي انخفاضاً يقارب 34%. والأهم من الرقم المجرد هو فهم السبب: ارتفاع الفائدة ولو بمقدار نصف نقطة مئوية لا يُقلص القدرة الشرائية بالنسبة ذاتها، بل قد يُقلص قيمة العقار الذي يستطيع المشتري تمويله بما يتراوح بين 4% و6%، وهذا يعني أن أثره الفعلي على الطلب أعمق مما يبدو. على شركات التطوير العقاري استيعاب هذه المعطيات جيداً، ومراجعة استراتيجيات التسعير بمرونة تتناسب مع المرحلة، لأن السوق الذكي من يقرأ الأرقام قبل أن تُقرأ عليه.</t>
+  </si>
+  <si>
+    <t>قانوني وتنظيمي</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍كل التوفيق لكم أبا عبدالعزيز
+▪️المركز في 10 نقاط:
+1️⃣ يرسم سياسات شمولية
+2️⃣ يرتبط بمجلس الوزراء
+3️⃣ رقابي على رقابة التفتيش
+4️⃣ رفع انتاجية الجهات التفتيشية
+5️⃣ معالجة الازدواجية الحكومية
+6️⃣ رفع الامتثال للأنظمة واللوائح
+7️⃣ تطوير لوائح التفتيش والرقابة
+8️⃣ ضبط تكاليف التفتيش والرقابة
+9️⃣ تحسين بيئة الأعمال بـ 🇸🇦
+🔟 المركز مولد لا محل للوطائف</t>
+  </si>
+  <si>
+    <t>إنشاء المركز الوطني للرقابة والتفتيش خطوة تنظيمية بالغة الأثر على بيئة الأعمال في المملكة، ومنها القطاع العقاري مباشرة. المركز يضع السياسات الشاملة للرقابة، ويرتبط بمجلس الوزراء مما يمنحه صلاحيات عليا، ويعمل على معالجة الازدواجية بين الجهات الحكومية وتخفيض تكاليف التفتيش ورفع مستوى الامتثال للأنظمة واللوائح. للمستثمر العقاري، هذا يعني بيئة أكثر شفافية وأقل تعقيداً إجرائياً، مما يعزز الثقة في السوق ويُسهم في استقطاب الاستثمارات وتسريع وتيرة المشاريع العقارية ضمن منظومة رؤية 2030.</t>
+  </si>
+  <si>
+    <t>٣١‏/٥‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍نسب الفائدة على التمويل مرتفعة لذا نوصي بـ الدمج لمن يستطيع لتحقيق:
+1️⃣ أعلى قيمة تمويل
+2️⃣ أقل هامش أرباح
+3️⃣ أفضل نسبة استقطاع
+ـ الطريقة: 👇
+📍دمج التمويل لأجل تملك العقار:
+▪️دمج العقاري مع الشخصي
+▪️أول 5 سنوات استقطاع 66%
+▪️الـ15 سنة التالية استقطاع 33%
+📍قيمة العقار المستحق:
+"حسب نسبة الفائدة البنكية"
+1️⃣ راتبك × 59 (أسوء سيناريو)
+2️⃣ راتبك × 69 (أفضل سيناريو)
+3️⃣ راتبك × 64 (سيناريو مثالي)
+* ينطبق على أغلب حالات التمويل
+* ينطبق على أغلب حالات الرواتب</t>
+  </si>
+  <si>
+    <t>في ظل ارتفاع نسب الفائدة على التمويل العقاري، يُعدّ دمج التمويل العقاري مع الشخصي من أذكى الخيارات المتاحة للمشتري الجاد، إذ يتيح له الحصول على أعلى قيمة تمويل ممكنة بأقل هامش أرباح وأفضل نسبة استقطاع. آلية الدمج تقوم على استقطاع 66% من الراتب خلال السنوات الخمس الأولى، ثم تنخفض إلى 33% في السنوات الخمس عشرة التالية. أما تقدير قيمة العقار الذي يستحقه المشتري فيحتسب بضرب الراتب الشهري في معامل يتراوح بين 59 في أضعف الحالات و69 في أفضلها، فيما يُمثّل المعامل 64 السيناريو الأنسب لأغلب حالات التمويل والرواتب. معرفة هذه الأرقام قبل التفاوض تمنحك موقفاً أقوى وقراراً أكثر رشداً.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍الوساطة العقارية كلها خير 
+▪️فيها فرص كبيرة للتوسع دون جهد إضافي، وبفضل الله، استفدت كثيرا من هذا المجال، لم أكن أحلم بذلك يوما 
+1️⃣ كن وسيطا تمويليًا
+2️⃣ كن وسيطا للمكاتب الهندسية
+3️⃣ كن وسيطا لمكاتب المحاماة
+4️⃣ كن وسيطا لشركات المقاولات
+5️⃣ كن وسيطا لأعمال نقل الملكية
+6️⃣ كن وسيطا لوكلاء والإعلانات
+▪️أعرف من علية القوم، يعملون وسطاء في المجالات المذكورة أعلاه
+▪️يفضل أن تفصح عن أعمال الوساطة عند التوصية بطريقة سلسة مع من سترتبط به بشكل محدود أو عرضي لمرة واحدة، ومنفتحاً بوضوح مع من تعمل معهم دائماً وعلاقتك بهم وثيقة ومستدامة، ولا تكن وسيطاً لما ذكر أعلاه إلا ما ترضاه لنفسك
+ ،،،
+ـ اجتهدوا واصبروا وتفائلوا
+ـ اللهم ارزقنا بالمد لا بالكد والله من وراء القصد</t>
+  </si>
+  <si>
+    <t>الوساطة العقارية من أذكى أدوات التوسع في هذا القطاع، إذ تتيح لك تحقيق دخل إضافي دون الحاجة إلى رأس مال ضخم. فالوسيط الناجح لا يقتصر على بيع العقارات وشرائها، بل يمتد دوره ليشمل التوسط في التمويل العقاري، وربط العملاء بالمكاتب الهندسية وشركات المقاولات ومكاتب المحاماة وخدمات نقل الملكية. والأهم في هذا العمل هو الشفافية، فأفصح عن علاقتك بمن توصي به، والتزم بتقديم ما ترضاه لنفسك فقط، لأن سمعتك هي رأس مالك الحقيقي في السوق العقاري. ابنِ شبكة علاقاتك بوعي، واجعل الثقة أساس كل توصية.</t>
+  </si>
+  <si>
+    <t>٢٨‏/٥‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍هذه رواية رجالها ثقات
+▪️أحد الرواة أبو سعد رضي الله عنه
+▪️الرواية:
+ـ دراسة لإنشاء هذا الجسر ويعني ذلك أن سكان حي سدرة على بعد 180 متر من المسار الرياضي وعلى بعد 4 كليو من:
+ـ حديقة الملك عبدالعزيز
+ـ محطة المترو
+ـ مقر أكسبو
+📍تعقيب:
+▪️المسار الرياضي الذي يقع بين جامعة الأميرة نورة و مركز كابسارك من أفضل المسارات في تقدري الشخصي، وقابل لرفع الكفاءة التشغيلية له رياضياً وسياحياً ومروياً نظراً لطبيعة الطريق والمنطقة المحيطة به وخلوه من الملكيات الخاصة</t>
+  </si>
+  <si>
+    <t>من المؤشرات التي يجدر بالمستثمر العقاري متابعتها: دراسات البنية التحتية المرتبطة بالأحياء الناشئة. حي سدرة في الرياض نموذج يستحق الرصد، إذ تشير المعطيات إلى وجود دراسة لإنشاء جسر يربطه بمسار رياضي متميز يقع بين جامعة الأميرة نورة ومركز كابسارك، وهو مسار يتميز بامتداده الطبيعي وخلوه من الملكيات الخاصة مما يجعله قابلاً للتطوير رياضياً وسياحياً. يُضاف إلى ذلك قرب الحي من حديقة الملك عبدالعزيز ومحطة المترو ومقر إكسبو بمسافة لا تتجاوز أربعة كيلومترات. وقاعدة عقارية راسخة تقول: إن مشاريع البنية التحتية تسبق ارتفاع الأسعار لا تتبعه، ومن يقرأ المؤشرات مبكراً يملك أفضلية حقيقية في السوق.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍يقول ابن القيم 
+▪️من رفق بعباد الله رفق الله به
+▪️ومن رحمهم رحمه الله
+▪️ومن أحسن إليهم أحسن الله إليه
+▪️ومن جاد عليهم جاد الله عليه
+▪️ومن نفعهم نفعه الله
+▪️ومن سترهم ستره الله
+▪️ومن عامل خلقه بصفة عامله الله بتلك الصفة بعينها في الدنيا والآخر</t>
+  </si>
+  <si>
+    <t>علّمنا ابن القيم رحمه الله أن معاملة الناس بالرفق والإحسان تعود على صاحبها بالخير المضاعف، وهذا المبدأ الراسخ هو جوهر العلاقة الصحية بين المطوّر والمشتري في السوق العقاري. المشتري الذي يُعامَل بالشفافية والأمانة يصبح سفيراً للمطوّر، والمطوّر الذي يُسلّم في موعده ويفي بالتزاماته يبني سمعة لا تقدّر بثمن. العقار الناجح لا يُبنى بالطوب والإسمنت فحسب، بل بحسن المعاملة وصدق الوعد.</t>
+  </si>
+  <si>
+    <t>٢٦‏/٥‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">شكرا لإثرائكم شيخنا
+▪️العمل على قضايا نزع العقارات تحتاج إلى فهم متين وقلم رصين وبناء للتسبيب يقطع الشك باليقين وهذا حمل يحمله المحامي القوي الأمين
+▪️فيمكن إدراك ما أمكن إدراكه من أن الضرر قد يقع على عقارات غير منزوعة نتج ضررها من نزع العقارات التي حولها أو وضع اليد عليها
+▪️ما يجب إدراكه كان ما كان أن الضرر قد يكون ناتجاً عن نزع جزء من العقار فيحدث ضررا أكبر في غير المنزوع وهذا من أسهل ما يمكن القيام به، ويحبكها الموفق في تسبيب بديع
+▪️ما لا يدرك كله ولا يكتب جله ولا يضبط محتمله، أن أغلب عقود أجور المنفعة لا تقيد كلفة وحسبة العوض على البناء لصالح المنتفع به، إذا كان هو المشيد للبناء وانتفع بجزء من المدة ثم نزع العقار، هذا فيه من التعقيد كحبل عقد في قتاد ومن عقلها فكأنما فك من عقال</t>
+  </si>
+  <si>
+    <t>قضايا نزع ملكية العقارات من أدق المسائل القانونية التي تستوجب إلماماً عميقاً بأحكام نظام نزع الملكية للمنفعة العامة، إذ لا يقتصر الضرر على العقار المنزوع وحده، بل قد يمتد أثره إلى العقارات المجاورة التي تتأثر قيمتها وانتفاعها جراء النزع. بل إن نزع جزء من العقار قد يُلحق ضرراً بالغاً بالجزء الباقي يفوق قيمة ما نُزع، وهذا حق للمالك يستوجب المطالبة به والتعويض عنه. ومن أخفى مسائل هذا الباب ما يتعلق بعقود الإيجار والبناء على الوجه المؤجر حين ينتفع المستأجر ببنائه جزءاً من المدة ثم يُنزع العقار، إذ تتشعب حسابات العوض بين المالك والمستأجر وتتعقد تقدير التعويض العادل لكل طرف. لذا فإن صاحب العقار المتضرر يحتاج إلى محامٍ متخصص يُحسن تسبيب مطالباته ويستوفي حقوقه كاملة.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍الانتقائية (Selectivity)
+▪️مساحة الوحدة: 40م²
+▪️الوحدة بالطابق الأول
+▪️موقف السيارة بالطابق الأرضي
+▪️السعر: 599,000﷼
+▪️سعر المتر²: 14,975﷼
+▪️نموذج البيع: على الخارطة
+▪️الموقع: حي السليمانية
+📍الرأي:
+▪️بعض الوحدات في الأبراج تجدها في الطابق الأرضي، لكن موقف السيارة في الطابق الخامس تحت الأرض، فتجربة الوصول لموقف السيارة غير مثالية
+▪️لهذا قد تكون الوحدة المرفقة خيارا أفضل من حيث المفاضلة لا من حيث التوصية، مقارنة ببعض المواقع التي تخطى المتر² فيها 18,000﷼
+▪️الاستثمار في الوحدات السكنية في الأبراج ليس شرطا أن تكون خيارا أفضل، فقد تكون وحدة سكنية على شارع 36 أفضل، والترويج أن الاستثمار في الأبراج خيار أفضل مطلقًا لا يمكن الاتفاق معه، لكن في المجمل العقارات في المواقع ذات الطلب العالي تغطي على أغلب العيوب، وعليه متى ما أخذت أفصل عقار في أفضل موقع بأفضل سعر فأنت حققت الانتقائية (Selectivity)</t>
+  </si>
+  <si>
+    <t>الانتقائية في العقار لا تعني اختيار الأغلى أو الأعلى، بل تعني الموازنة الذكية بين السعر والموقع وجودة التجربة السكنية. وحدة بمساحة 40 متراً في حي السليمانية بسعر متر يقارب 15,000 ريال، مع موقف سيارة في الطابق الأول، قد تتفوق عملياً على وحدة في برج فارهٍ يشترط قطع خمسة طوابق تحت الأرض للوصول إلى سيارتك. كذلك لا ينبغي تعميم أن الاستثمار في الأبراج دائماً هو الخيار الأمثل، فوحدة سكنية على شارع رئيسي واسع قد تحقق عوائد وراحة أفضل. المبدأ الذهبي في الانتقائية العقارية هو: حين تجد عقاراً في موقع ذي طلب مرتفع بسعر عادل وتفاصيل مدروسة، فأنت أمام فرصة حقيقية لا مجرد صفقة.</t>
+  </si>
+  <si>
+    <t>٢٥‏/٥‏/٢٠٢٦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">📍تجربة مدير الحي (NHM)
+"مدير حي سدرة: فهد البريه"
+،،،
+▪️المجتمعات السكنية المتكاملة توفر وظائف عالية المستوى والدخل 
+▪️التكلفة يتحملها السكان لكن بتكلفة أقل نظراً لتعددية الوحدات
+▪️خلق الاستدامة ورسم السياسة التشغيلية المتكاملة هو نتيجة الشركات التطوير العقاري الضخمة
+▪️إن أهم أثر قانوني هو القدرة على استراد الحق في أقصر وقت وأقل جهد
+▪️التعامل مع الشركات الضخمة يعني بقائها عقود من الزمن بوعاء مالي ضخم يستوعب حفظ وضمان الحقوق
+▪️سعيد بـ :
+ـ كوادر وطنية ذو كفاءة
+ـ إدارة حي تدار بعمل مؤسسي
+ـ لطافة و طرافة و طمئانية مع 👇</t>
+  </si>
+  <si>
+    <t>المجتمعات السكنية المتكاملة ليست مجرد مساكن، بل منظومة حياة متكاملة تخلق فرص عمل راقية وتوزع التكاليف التشغيلية على السكان بصورة عادلة تخفف العبء الفردي. شركات التطوير العقاري الكبرى تتميز بقدرتها على بناء سياسات تشغيلية مستدامة وحماية حقوق الملاك لعقود طويلة بفضل ملاءتها المالية الضخمة، مما يمنح المقيم ضماناً حقيقياً واسترداداً سريعاً لحقوقه عند الحاجة. اختيار المطور الكبير ذي السمعة الراسخة ليس ترفاً، بل قرار استثماري واعٍ يصون حقوقك ويرفع جودة حياتك.</t>
+  </si>
+  <si>
     <t>حساب المصدر</t>
   </si>
   <si>
@@ -60,9 +405,6 @@
   </si>
   <si>
     <t>تاريخ الاستخراج</t>
-  </si>
-  <si>
-    <t>٧‏/٦‏/٢٠٢٦</t>
   </si>
   <si>
     <t>إجمالي التغريدات</t>
@@ -75,7 +417,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -88,8 +430,12 @@
       <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF198754"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -99,6 +445,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F7FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -114,10 +470,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -508,6 +880,606 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4"/>
+      <c r="I2" s="2">
+        <v>30</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="6">
+        <v>8</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="I3">
+        <v>117</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="I4" s="2">
+        <v>6</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="6">
+        <v>8</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="7"/>
+      <c r="I5">
+        <v>24</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3">
+        <v>9</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="I6" s="2">
+        <v>58</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="6">
+        <v>8</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="I7">
+        <v>27</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3">
+        <v>8</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="4"/>
+      <c r="I8" s="2">
+        <v>42</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="6">
+        <v>8</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="7"/>
+      <c r="I9">
+        <v>73</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="3">
+        <v>8</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="I10" s="2">
+        <v>5</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="6">
+        <v>8</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="7"/>
+      <c r="I11">
+        <v>63</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="3">
+        <v>8</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="I12" s="2">
+        <v>70</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="6">
+        <v>8</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="7"/>
+      <c r="I13">
+        <v>52</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="3">
+        <v>8</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="I14" s="2">
+        <v>6</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="6">
+        <v>8</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G15" s="7"/>
+      <c r="I15">
+        <v>402</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="3">
+        <v>8</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="I16" s="2">
+        <v>179</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="6">
+        <v>8</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" s="7"/>
+      <c r="I17">
+        <v>108</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="3">
+        <v>8</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="I18" s="2">
+        <v>16</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="6">
+        <v>8</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="7"/>
+      <c r="I19">
+        <v>17</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="3">
+        <v>8</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="4"/>
+      <c r="I20" s="2">
+        <v>86</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="6">
+        <v>8</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G21" s="7"/>
+      <c r="I21">
+        <v>114</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -516,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -525,34 +1497,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -560,7 +1532,39 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>